<commit_message>
Upload latest Excel dashboard
</commit_message>
<xml_diff>
--- a/Excel DashBoard Project.xlsx
+++ b/Excel DashBoard Project.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sales_Data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -341,145 +341,7 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="48">
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
     </dxf>
@@ -21658,186 +21520,153 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100">
-              <a:ln>
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-              </a:ln>
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>1</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-IN" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </a:rPr>
-            <a:t>By using the "Dashboard" option, we can analyze product sales, total sales, and total unit sales based on month, place, and product.</a:t>
+            <a:t>1."This dashboard analyzes product sales, total sales amount, and total units sold using interactive filters. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>2.</a:t>
+            <a:t>2.The </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-IN" b="1">
+            <a:rPr lang="en-IN" sz="1500" b="1">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>"Product" is useful for analyzing "Top 3 product sales," "Bottom 3 product sales," and "Product units" based on month, place, and product.</a:t>
+            <a:t>Dashboard</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1500">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> page provides an overview of sales by month, product, and place. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </a:rPr>
-            <a:t>3.</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-IN" b="1">
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>In this "Product" section, we cannot apply product-wise sales. We can only see "Top 3 sales products" and "Bottom 3 sales products."</a:t>
+            <a:t>3.The </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1500" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Product</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1500">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> page highlights the Top 3 and Bottom 3 selling products. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>4.</a:t>
+            <a:t>4.The </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-IN" b="1">
+            <a:rPr lang="en-IN" sz="1500" b="1">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>"Sales Man" is useful for analyzing "Top 3 sales by salesman," "Bottom 3 sales by salesman," and the total performance of salesmen.</a:t>
+            <a:t>Sales Man</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1500">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> page analyzes salesperson performance, including the Top 3 and Bottom 3 performers. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>5.</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-IN" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>The Dashboard is useful for analyzing "Product Sales" and "Sales Man Performance."</a:t>
+            <a:t>5.Interactive slicers allow users to filter data by date, product, and location. </a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-              <a:ln w="0"/>
+            <a:rPr lang="en-IN" sz="1500">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>6.</a:t>
+            <a:t>6.This project was developed using Microsoft Excel 2016.</a:t>
           </a:r>
-          <a:r>
-            <a:rPr lang="en-IN" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>"I used Excel 2016 version for this project."</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
+          <a:endParaRPr lang="en-IN" sz="1500" b="1" cap="none" spc="0">
             <a:ln w="0"/>
             <a:solidFill>
               <a:schemeClr val="tx1"/>
@@ -21849,22 +21678,9 @@
                 </a:schemeClr>
               </a:outerShdw>
             </a:effectLst>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-IN" sz="1100" b="1" cap="none" spc="0">
-            <a:ln w="0"/>
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst>
-              <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                <a:schemeClr val="dk1">
-                  <a:alpha val="40000"/>
-                </a:schemeClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
       </xdr:txBody>
@@ -24806,8 +24622,157 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="26">
-  <location ref="A67:B74" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable13" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+  <location ref="A1:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisRow" numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="0"/>
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="13">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="3" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="33">
+  <location ref="A91:B95" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField numFmtId="14" showAll="0">
       <items count="15">
@@ -24828,8 +24793,18 @@
         <item t="default" sd="0"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="7">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
       <items count="7">
         <item x="2"/>
         <item x="0"/>
@@ -24875,18 +24850,9 @@
     </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="2"/>
+    <field x="1"/>
   </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
+  <rowItems count="4">
     <i>
       <x v="3"/>
     </i>
@@ -24906,7 +24872,7 @@
   <dataFields count="1">
     <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="2">
+  <chartFormats count="6">
     <chartFormat chart="20" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -24925,8 +24891,53 @@
         </references>
       </pivotArea>
     </chartFormat>
+    <chartFormat chart="24" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="28" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="30" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="32" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="1" type="count" evalOrder="-1" id="2" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 top="0" val="3" filterVal="3"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -24935,8 +24946,184 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable16" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
+<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="35">
+  <location ref="A82:B86" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" measureFilter="1">
+      <items count="7">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="20" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="22" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="24" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="30" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="32" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="34" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="1" type="count" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="3" filterVal="3"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable16" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
   <location ref="A39:A40" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="9">
     <pivotField numFmtId="14" showAll="0">
@@ -25014,7 +25201,7 @@
     <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0" numFmtId="3"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="47">
+    <format dxfId="0">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -25083,8 +25270,193 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="42">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable7" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="31">
+  <location ref="A98:B105" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="7">
+    <chartFormat chart="20" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="22" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="24" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="26" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="27" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="28" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="30" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="42">
   <location ref="A55:B59" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField numFmtId="14" showAll="0">
@@ -25339,8 +25711,286 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable14" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
+  <location ref="A18:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="3" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="26">
+  <location ref="A67:B74" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="20" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="22" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17">
   <location ref="A43:A44" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="9">
     <pivotField numFmtId="14" showAll="0">
@@ -25418,7 +26068,7 @@
     <dataField name="Count of Amount" fld="6" subtotal="count" baseField="0" baseItem="1550835536" numFmtId="3"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="46">
+    <format dxfId="1">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -25487,8 +26137,174 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34">
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable15" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19">
+  <location ref="A29:B36" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="3" showAll="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="3" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="14" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34">
   <location ref="A47:B51" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField numFmtId="14" showAll="0">
@@ -25710,1006 +26526,6 @@
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
     <filter fld="2" type="count" evalOrder="-1" id="2" iMeasureFld="0">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <top10 val="3" filterVal="3"/>
-        </filterColumn>
-      </autoFilter>
-    </filter>
-  </filters>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable13" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="A1:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisRow" numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="0"/>
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="13">
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="3" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="31">
-  <location ref="A98:B105" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="4"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="7">
-    <chartFormat chart="20" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="22" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="24" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="26" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="27" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="28" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="30" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable14" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A18:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="3" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable15" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19">
-  <location ref="A29:B36" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="3" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="14" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="33">
-  <location ref="A91:B95" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0" measureFilter="1">
-      <items count="7">
-        <item x="4"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="20" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="22" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="24" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="28" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="30" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="32" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="1">
-    <filter fld="1" type="count" evalOrder="-1" id="2" iMeasureFld="0">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <top10 top="0" val="3" filterVal="3"/>
-        </filterColumn>
-      </autoFilter>
-    </filter>
-  </filters>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="35">
-  <location ref="A82:B86" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item t="default" sd="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0" measureFilter="1">
-      <items count="7">
-        <item x="4"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="6">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Units" fld="5" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="20" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="22" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="24" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="30" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="32" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="34" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="1">
-    <filter fld="1" type="count" evalOrder="-1" id="1" iMeasureFld="0">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <top10 val="3" filterVal="3"/>

</xml_diff>